<commit_message>
Major updates to ACS data pull script, started to incorporate CPS data from Censu Bureau
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/CPI Inflation Adjustment Factors.xlsx
+++ b/Indicator_Gen/config/CPI Inflation Adjustment Factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F2BDD74-D3EB-4C2F-8515-813FEFE541F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E33722AB-E14C-428C-9DEF-00ACA87EE150}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="7" r:id="rId1"/>
@@ -161,14 +161,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -429,15 +426,15 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -746,18 +743,18 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -765,7 +762,7 @@
       <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2669,7 +2666,7 @@
         <f t="shared" si="3"/>
         <v>1.1976131001942825</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8">
         <f t="shared" si="4"/>
         <v>1.1079655842353593</v>
       </c>
@@ -3821,7 +3818,7 @@
         <f t="shared" si="3"/>
         <v>1.2189347486437045</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8">
         <f t="shared" si="4"/>
         <v>1.1285870188193361</v>
       </c>

</xml_diff>

<commit_message>
Testing minor changes with readme updates
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/CPI Inflation Adjustment Factors.xlsx
+++ b/Indicator_Gen/config/CPI Inflation Adjustment Factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BFBC93F-15CC-4E8A-B56A-2E518D94D37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2190DFB8-25DB-4A54-AA59-34CFA01B2EF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="7" r:id="rId1"/>

</xml_diff>

<commit_message>
Final cleaning/reorganization of 2024, reduced file size of all configuration files
</commit_message>
<xml_diff>
--- a/Indicator_Gen/config/CPI Inflation Adjustment Factors.xlsx
+++ b/Indicator_Gen/config/CPI Inflation Adjustment Factors.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfontes\Documents\Projects\Regional-Monitoring\Indicator_Gen\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92AD5063-4570-4281-949D-EFD520465851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC6CAF0D-8AAE-4F73-AB21-285F32C62284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-90" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sources" sheetId="7" r:id="rId1"/>

</xml_diff>